<commit_message>
Record the final 2026-27 Vegas win totals
Final consensus pull on October 13, 2026, one week before the October 20
opener. Updates picks.xlsx and projections.csv and adds the all-books
snapshot; seven lines moved by one game since the October 2 preview.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0176YHQyKixwwmKjCn6TPHrC
</commit_message>
<xml_diff>
--- a/nba-over-under-2026-2027/picks.xlsx
+++ b/nba-over-under-2026-2027/picks.xlsx
@@ -644,7 +644,7 @@
         <v>35</v>
       </c>
       <c r="C3" t="n">
-        <v>50.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="4">
@@ -666,7 +666,7 @@
         <v>35</v>
       </c>
       <c r="C5" t="n">
-        <v>39.5</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="6">
@@ -699,7 +699,7 @@
         <v>35</v>
       </c>
       <c r="C8" t="n">
-        <v>49.5</v>
+        <v>48.5</v>
       </c>
     </row>
     <row r="9">
@@ -721,7 +721,7 @@
         <v>35</v>
       </c>
       <c r="C10" t="n">
-        <v>45.5</v>
+        <v>46.5</v>
       </c>
     </row>
     <row r="11">
@@ -820,7 +820,7 @@
         <v>36</v>
       </c>
       <c r="C19" t="n">
-        <v>38.5</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="20">
@@ -831,7 +831,7 @@
         <v>36</v>
       </c>
       <c r="C20" t="n">
-        <v>47.5</v>
+        <v>48.5</v>
       </c>
     </row>
     <row r="21">
@@ -897,7 +897,7 @@
         <v>36</v>
       </c>
       <c r="C26" t="n">
-        <v>61.5</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="27">

</xml_diff>